<commit_message>
data: hourly update 2026-07-12 23:05Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-12.xlsx
+++ b/data/output/workbook/2026-07-12.xlsx
@@ -581,7 +581,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="10839450"/>
+    <ext cx="10125075" cy="10582275"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -611,7 +611,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="10496550"/>
+    <ext cx="10125075" cy="10648950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-12 18:01</t>
+          <t>2026-07-12 19:04</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q83"/>
+  <dimension ref="A1:Q81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5843,167 +5843,325 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="29" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians offense vs Miami Marlins defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B68" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C68" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D68" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E68" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F68" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G68" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H68" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I68" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J68" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K68" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L68" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M68" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N68" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O68" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P68" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q68" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
     <row r="69">
-      <c r="A69" s="29" t="inlineStr">
-        <is>
-          <t>Cleveland Guardians offense vs Miami Marlins defense</t>
+      <c r="A69" s="31" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B69" s="32" t="n">
+        <v>3.919</v>
+      </c>
+      <c r="C69" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D69" s="32" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="E69" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F69" s="32" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G69" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H69" s="34" t="inlineStr">
+        <is>
+          <t>25th</t>
+        </is>
+      </c>
+      <c r="I69" s="32" t="inlineStr"/>
+      <c r="J69" s="36" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="K69" s="32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L69" s="32" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="M69" s="32" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="N69" s="32" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="O69" s="32" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="P69" s="32" t="n">
+        <v>4.271</v>
+      </c>
+      <c r="Q69" s="35" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B70" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C70" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D70" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E70" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F70" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G70" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H70" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I70" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J70" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K70" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L70" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M70" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N70" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O70" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P70" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q70" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A70" s="31" t="inlineStr">
+        <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B70" s="32" t="n">
+        <v>7.735</v>
+      </c>
+      <c r="C70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H70" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I70" s="32" t="inlineStr"/>
+      <c r="J70" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P70" s="32" t="n">
+        <v>7.694</v>
+      </c>
+      <c r="Q70" s="35" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>3.919</v>
-      </c>
-      <c r="C71" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="D71" s="32" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="E71" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="F71" s="32" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="G71" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="H71" s="34" t="inlineStr">
-        <is>
-          <t>25th</t>
+        <v>0.959</v>
+      </c>
+      <c r="C71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="I71" s="32" t="inlineStr"/>
-      <c r="J71" s="36" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="K71" s="32" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="L71" s="32" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="M71" s="32" t="n">
-        <v>4.267</v>
-      </c>
-      <c r="N71" s="32" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="O71" s="32" t="n">
-        <v>3.8</v>
+      <c r="J71" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="P71" s="32" t="n">
-        <v>4.271</v>
+        <v>1.082</v>
       </c>
       <c r="Q71" s="35" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B72" s="32" t="n">
-        <v>7.735</v>
+        <v>8</v>
       </c>
       <c r="C72" s="32" t="inlineStr">
         <is>
@@ -6067,392 +6225,392 @@
         </is>
       </c>
       <c r="P72" s="32" t="n">
-        <v>7.694</v>
+        <v>8.531000000000001</v>
       </c>
       <c r="Q72" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B73" s="32" t="n">
-        <v>0.959</v>
-      </c>
-      <c r="C73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H73" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>0.494</v>
+      </c>
+      <c r="C73" s="32" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="D73" s="32" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E73" s="32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F73" s="32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G73" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="34" t="inlineStr">
+        <is>
+          <t>29th</t>
         </is>
       </c>
       <c r="I73" s="32" t="inlineStr"/>
-      <c r="J73" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J73" s="36" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="K73" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M73" s="32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N73" s="32" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O73" s="32" t="n">
+        <v>0.333</v>
       </c>
       <c r="P73" s="32" t="n">
-        <v>1.082</v>
+        <v>0.578</v>
       </c>
       <c r="Q73" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="31" t="inlineStr">
-        <is>
-          <t>Batter K/G</t>
-        </is>
-      </c>
-      <c r="B74" s="32" t="n">
-        <v>8</v>
-      </c>
-      <c r="C74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H74" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I74" s="32" t="inlineStr"/>
-      <c r="J74" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P74" s="32" t="n">
-        <v>8.531000000000001</v>
-      </c>
-      <c r="Q74" s="35" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="31" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B75" s="32" t="n">
-        <v>0.494</v>
-      </c>
-      <c r="C75" s="32" t="n">
-        <v>0.267</v>
-      </c>
-      <c r="D75" s="32" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E75" s="32" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F75" s="32" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G75" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H75" s="34" t="inlineStr">
-        <is>
-          <t>29th</t>
-        </is>
-      </c>
-      <c r="I75" s="32" t="inlineStr"/>
-      <c r="J75" s="36" t="inlineStr">
+      <c r="A75" s="29" t="inlineStr">
+        <is>
+          <t>Miami Marlins offense vs Cleveland Guardians defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B76" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D76" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E76" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F76" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G76" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H76" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I76" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J76" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K76" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L76" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M76" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N76" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O76" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P76" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q76" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="31" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B77" s="32" t="n">
+        <v>4.647</v>
+      </c>
+      <c r="C77" s="32" t="n">
+        <v>5.367</v>
+      </c>
+      <c r="D77" s="32" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="E77" s="32" t="n">
+        <v>5.867</v>
+      </c>
+      <c r="F77" s="32" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="G77" s="32" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H77" s="33" t="inlineStr">
+        <is>
+          <t>20th</t>
+        </is>
+      </c>
+      <c r="I77" s="32" t="inlineStr"/>
+      <c r="J77" s="36" t="inlineStr">
         <is>
           <t>3rd</t>
         </is>
       </c>
-      <c r="K75" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L75" s="32" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M75" s="32" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N75" s="32" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="O75" s="32" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="P75" s="32" t="n">
-        <v>0.578</v>
-      </c>
-      <c r="Q75" s="35" t="inlineStr">
-        <is>
-          <t>Opp 1st Inn R/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="29" t="inlineStr">
-        <is>
-          <t>Miami Marlins offense vs Cleveland Guardians defense</t>
+      <c r="K77" s="32" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L77" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M77" s="32" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N77" s="32" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="O77" s="32" t="n">
+        <v>4.133</v>
+      </c>
+      <c r="P77" s="32" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="Q77" s="35" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B78" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C78" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D78" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E78" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F78" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G78" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H78" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I78" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J78" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K78" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L78" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M78" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N78" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O78" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P78" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q78" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A78" s="31" t="inlineStr">
+        <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B78" s="32" t="n">
+        <v>8.286</v>
+      </c>
+      <c r="C78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H78" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I78" s="32" t="inlineStr"/>
+      <c r="J78" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P78" s="32" t="n">
+        <v>7.939</v>
+      </c>
+      <c r="Q78" s="35" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B79" s="32" t="n">
-        <v>4.647</v>
-      </c>
-      <c r="C79" s="32" t="n">
-        <v>5.367</v>
-      </c>
-      <c r="D79" s="32" t="n">
-        <v>5.45</v>
-      </c>
-      <c r="E79" s="32" t="n">
-        <v>5.867</v>
-      </c>
-      <c r="F79" s="32" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="G79" s="32" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="H79" s="33" t="inlineStr">
-        <is>
-          <t>20th</t>
+        <v>0.918</v>
+      </c>
+      <c r="C79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="I79" s="32" t="inlineStr"/>
-      <c r="J79" s="36" t="inlineStr">
-        <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="K79" s="32" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="L79" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="M79" s="32" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="N79" s="32" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="O79" s="32" t="n">
-        <v>4.133</v>
+      <c r="J79" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="P79" s="32" t="n">
-        <v>4.07</v>
+        <v>1.143</v>
       </c>
       <c r="Q79" s="35" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B80" s="32" t="n">
-        <v>8.286</v>
+        <v>7.816</v>
       </c>
       <c r="C80" s="32" t="inlineStr">
         <is>
@@ -6516,226 +6674,68 @@
         </is>
       </c>
       <c r="P80" s="32" t="n">
-        <v>7.939</v>
+        <v>9.388</v>
       </c>
       <c r="Q80" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B81" s="32" t="n">
-        <v>0.918</v>
-      </c>
-      <c r="C81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H81" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>0.578</v>
+      </c>
+      <c r="C81" s="32" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="D81" s="32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E81" s="32" t="n">
+        <v>0.733</v>
+      </c>
+      <c r="F81" s="32" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G81" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" s="34" t="inlineStr">
+        <is>
+          <t>21st</t>
         </is>
       </c>
       <c r="I81" s="32" t="inlineStr"/>
-      <c r="J81" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J81" s="33" t="inlineStr">
+        <is>
+          <t>12th</t>
+        </is>
+      </c>
+      <c r="K81" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M81" s="32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N81" s="32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O81" s="32" t="n">
+        <v>0.433</v>
       </c>
       <c r="P81" s="32" t="n">
-        <v>1.143</v>
+        <v>0.361</v>
       </c>
       <c r="Q81" s="35" t="inlineStr">
-        <is>
-          <t>Opp HR/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="31" t="inlineStr">
-        <is>
-          <t>Batter K/G</t>
-        </is>
-      </c>
-      <c r="B82" s="32" t="n">
-        <v>7.816</v>
-      </c>
-      <c r="C82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H82" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I82" s="32" t="inlineStr"/>
-      <c r="J82" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P82" s="32" t="n">
-        <v>9.388</v>
-      </c>
-      <c r="Q82" s="35" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="31" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B83" s="32" t="n">
-        <v>0.578</v>
-      </c>
-      <c r="C83" s="32" t="n">
-        <v>0.5669999999999999</v>
-      </c>
-      <c r="D83" s="32" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E83" s="32" t="n">
-        <v>0.733</v>
-      </c>
-      <c r="F83" s="32" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G83" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H83" s="34" t="inlineStr">
-        <is>
-          <t>21st</t>
-        </is>
-      </c>
-      <c r="I83" s="32" t="inlineStr"/>
-      <c r="J83" s="33" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="K83" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L83" s="32" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="M83" s="32" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N83" s="32" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="O83" s="32" t="n">
-        <v>0.433</v>
-      </c>
-      <c r="P83" s="32" t="n">
-        <v>0.361</v>
-      </c>
-      <c r="Q83" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -6754,7 +6754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q81"/>
+  <dimension ref="A1:Q82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6771,250 +6771,171 @@
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="29" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="29" t="inlineStr">
         <is>
           <t>Los Angeles Angels offense vs Minnesota Twins defense</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="30" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B68" s="30" t="inlineStr">
+      <c r="B69" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C68" s="30" t="inlineStr">
+      <c r="C69" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D68" s="30" t="inlineStr">
+      <c r="D69" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E68" s="30" t="inlineStr">
+      <c r="E69" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F68" s="30" t="inlineStr">
+      <c r="F69" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G68" s="30" t="inlineStr">
+      <c r="G69" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H68" s="30" t="inlineStr">
+      <c r="H69" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I68" s="30" t="inlineStr">
+      <c r="I69" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J68" s="30" t="inlineStr">
+      <c r="J69" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K68" s="30" t="inlineStr">
+      <c r="K69" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L68" s="30" t="inlineStr">
+      <c r="L69" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M68" s="30" t="inlineStr">
+      <c r="M69" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N68" s="30" t="inlineStr">
+      <c r="N69" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O68" s="30" t="inlineStr">
+      <c r="O69" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P68" s="30" t="inlineStr">
+      <c r="P69" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q68" s="30" t="inlineStr">
+      <c r="Q69" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B69" s="32" t="n">
-        <v>4.595</v>
-      </c>
-      <c r="C69" s="32" t="n">
-        <v>4.567</v>
-      </c>
-      <c r="D69" s="32" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="E69" s="32" t="n">
-        <v>4.067</v>
-      </c>
-      <c r="F69" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="G69" s="32" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="H69" s="36" t="inlineStr">
-        <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="I69" s="32" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J69" s="36" t="inlineStr">
-        <is>
-          <t>8th</t>
-        </is>
-      </c>
-      <c r="K69" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="L69" s="32" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="M69" s="32" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="N69" s="32" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="O69" s="32" t="n">
-        <v>5.167</v>
-      </c>
-      <c r="P69" s="32" t="n">
-        <v>4.976</v>
-      </c>
-      <c r="Q69" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B70" s="32" t="n">
-        <v>7.714</v>
-      </c>
-      <c r="C70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I70" s="32" t="inlineStr"/>
-      <c r="J70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>4.595</v>
+      </c>
+      <c r="C70" s="32" t="n">
+        <v>4.567</v>
+      </c>
+      <c r="D70" s="32" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="E70" s="32" t="n">
+        <v>4.067</v>
+      </c>
+      <c r="F70" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="G70" s="32" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="H70" s="36" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="I70" s="32" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J70" s="36" t="inlineStr">
+        <is>
+          <t>8th</t>
+        </is>
+      </c>
+      <c r="K70" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="L70" s="32" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="M70" s="32" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="N70" s="32" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="O70" s="32" t="n">
+        <v>5.167</v>
       </c>
       <c r="P70" s="32" t="n">
-        <v>8.305999999999999</v>
+        <v>4.976</v>
       </c>
       <c r="Q70" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>1.184</v>
+        <v>7.714</v>
       </c>
       <c r="C71" s="32" t="inlineStr">
         <is>
@@ -7078,22 +6999,22 @@
         </is>
       </c>
       <c r="P71" s="32" t="n">
-        <v>0.918</v>
+        <v>8.305999999999999</v>
       </c>
       <c r="Q71" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B72" s="32" t="n">
-        <v>9.286</v>
+        <v>1.184</v>
       </c>
       <c r="C72" s="32" t="inlineStr">
         <is>
@@ -7157,313 +7078,313 @@
         </is>
       </c>
       <c r="P72" s="32" t="n">
-        <v>8.265000000000001</v>
+        <v>0.918</v>
       </c>
       <c r="Q72" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
         <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B73" s="32" t="n">
+        <v>9.286</v>
+      </c>
+      <c r="C73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="inlineStr"/>
+      <c r="J73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P73" s="32" t="n">
+        <v>8.265000000000001</v>
+      </c>
+      <c r="Q73" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B73" s="32" t="n">
+      <c r="B74" s="32" t="n">
         <v>0.59</v>
       </c>
-      <c r="C73" s="32" t="n">
+      <c r="C74" s="32" t="n">
         <v>0.5669999999999999</v>
       </c>
-      <c r="D73" s="32" t="n">
+      <c r="D74" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="E73" s="32" t="n">
+      <c r="E74" s="32" t="n">
         <v>0.533</v>
       </c>
-      <c r="F73" s="32" t="n">
+      <c r="F74" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="G73" s="32" t="n">
+      <c r="G74" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="H73" s="33" t="inlineStr">
+      <c r="H74" s="33" t="inlineStr">
         <is>
           <t>11th</t>
         </is>
       </c>
-      <c r="I73" s="32" t="inlineStr"/>
-      <c r="J73" s="36" t="inlineStr">
+      <c r="I74" s="32" t="inlineStr"/>
+      <c r="J74" s="36" t="inlineStr">
         <is>
           <t>6th</t>
         </is>
       </c>
-      <c r="K73" s="32" t="n">
+      <c r="K74" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="L73" s="32" t="n">
+      <c r="L74" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="M73" s="32" t="n">
+      <c r="M74" s="32" t="n">
         <v>0.267</v>
       </c>
-      <c r="N73" s="32" t="n">
+      <c r="N74" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="O73" s="32" t="n">
+      <c r="O74" s="32" t="n">
         <v>0.367</v>
       </c>
-      <c r="P73" s="32" t="n">
+      <c r="P74" s="32" t="n">
         <v>0.554</v>
       </c>
-      <c r="Q73" s="35" t="inlineStr">
+      <c r="Q74" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="29" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="29" t="inlineStr">
         <is>
           <t>Minnesota Twins offense vs Los Angeles Angels defense</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="30" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B76" s="30" t="inlineStr">
+      <c r="B77" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C76" s="30" t="inlineStr">
+      <c r="C77" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D76" s="30" t="inlineStr">
+      <c r="D77" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E76" s="30" t="inlineStr">
+      <c r="E77" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F76" s="30" t="inlineStr">
+      <c r="F77" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G76" s="30" t="inlineStr">
+      <c r="G77" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H76" s="30" t="inlineStr">
+      <c r="H77" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I76" s="30" t="inlineStr">
+      <c r="I77" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J76" s="30" t="inlineStr">
+      <c r="J77" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K76" s="30" t="inlineStr">
+      <c r="K77" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L76" s="30" t="inlineStr">
+      <c r="L77" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M76" s="30" t="inlineStr">
+      <c r="M77" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N76" s="30" t="inlineStr">
+      <c r="N77" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O76" s="30" t="inlineStr">
+      <c r="O77" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P76" s="30" t="inlineStr">
+      <c r="P77" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q76" s="30" t="inlineStr">
+      <c r="Q77" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B77" s="32" t="n">
-        <v>4.807</v>
-      </c>
-      <c r="C77" s="32" t="n">
-        <v>5.467</v>
-      </c>
-      <c r="D77" s="32" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="E77" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="F77" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="G77" s="32" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="H77" s="34" t="inlineStr">
-        <is>
-          <t>22nd</t>
-        </is>
-      </c>
-      <c r="I77" s="32" t="inlineStr"/>
-      <c r="J77" s="33" t="inlineStr">
-        <is>
-          <t>20th</t>
-        </is>
-      </c>
-      <c r="K77" s="32" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="L77" s="32" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="M77" s="32" t="n">
-        <v>5.133</v>
-      </c>
-      <c r="N77" s="32" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="O77" s="32" t="n">
-        <v>4.633</v>
-      </c>
-      <c r="P77" s="32" t="n">
-        <v>5.131</v>
-      </c>
-      <c r="Q77" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B78" s="32" t="n">
-        <v>7.776</v>
-      </c>
-      <c r="C78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H78" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>4.807</v>
+      </c>
+      <c r="C78" s="32" t="n">
+        <v>5.467</v>
+      </c>
+      <c r="D78" s="32" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E78" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F78" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="G78" s="32" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H78" s="34" t="inlineStr">
+        <is>
+          <t>22nd</t>
         </is>
       </c>
       <c r="I78" s="32" t="inlineStr"/>
-      <c r="J78" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J78" s="33" t="inlineStr">
+        <is>
+          <t>20th</t>
+        </is>
+      </c>
+      <c r="K78" s="32" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="L78" s="32" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="M78" s="32" t="n">
+        <v>5.133</v>
+      </c>
+      <c r="N78" s="32" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="O78" s="32" t="n">
+        <v>4.633</v>
       </c>
       <c r="P78" s="32" t="n">
-        <v>8.244999999999999</v>
+        <v>5.131</v>
       </c>
       <c r="Q78" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B79" s="32" t="n">
-        <v>1.061</v>
+        <v>7.776</v>
       </c>
       <c r="C79" s="32" t="inlineStr">
         <is>
@@ -7527,22 +7448,22 @@
         </is>
       </c>
       <c r="P79" s="32" t="n">
-        <v>1.061</v>
+        <v>8.244999999999999</v>
       </c>
       <c r="Q79" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B80" s="32" t="n">
-        <v>8.939</v>
+        <v>1.061</v>
       </c>
       <c r="C80" s="32" t="inlineStr">
         <is>
@@ -7606,68 +7527,147 @@
         </is>
       </c>
       <c r="P80" s="32" t="n">
-        <v>8.816000000000001</v>
+        <v>1.061</v>
       </c>
       <c r="Q80" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
         <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B81" s="32" t="n">
+        <v>8.939</v>
+      </c>
+      <c r="C81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I81" s="32" t="inlineStr"/>
+      <c r="J81" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P81" s="32" t="n">
+        <v>8.816000000000001</v>
+      </c>
+      <c r="Q81" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B81" s="32" t="n">
+      <c r="B82" s="32" t="n">
         <v>0.6870000000000001</v>
       </c>
-      <c r="C81" s="32" t="n">
+      <c r="C82" s="32" t="n">
         <v>0.9330000000000001</v>
       </c>
-      <c r="D81" s="32" t="n">
+      <c r="D82" s="32" t="n">
         <v>0.85</v>
       </c>
-      <c r="E81" s="32" t="n">
+      <c r="E82" s="32" t="n">
         <v>0.9330000000000001</v>
       </c>
-      <c r="F81" s="32" t="n">
+      <c r="F82" s="32" t="n">
         <v>1.1</v>
       </c>
-      <c r="G81" s="32" t="n">
+      <c r="G82" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="H81" s="33" t="inlineStr">
+      <c r="H82" s="33" t="inlineStr">
         <is>
           <t>17th</t>
         </is>
       </c>
-      <c r="I81" s="32" t="inlineStr"/>
-      <c r="J81" s="33" t="inlineStr">
+      <c r="I82" s="32" t="inlineStr"/>
+      <c r="J82" s="33" t="inlineStr">
         <is>
           <t>18th</t>
         </is>
       </c>
-      <c r="K81" s="32" t="n">
+      <c r="K82" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="L81" s="32" t="n">
+      <c r="L82" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="M81" s="32" t="n">
+      <c r="M82" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="N81" s="32" t="n">
+      <c r="N82" s="32" t="n">
         <v>0.55</v>
       </c>
-      <c r="O81" s="32" t="n">
+      <c r="O82" s="32" t="n">
         <v>0.5669999999999999</v>
       </c>
-      <c r="P81" s="32" t="n">
+      <c r="P82" s="32" t="n">
         <v>0.578</v>
       </c>
-      <c r="Q81" s="35" t="inlineStr">
+      <c r="Q82" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -8902,10 +8902,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5876</v>
+        <v>0.5946</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-142</v>
+        <v>-147</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>178</v>
@@ -8932,7 +8932,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 58.8% (fair -142). Your call.</t>
+          <t>Model 59.5% (fair -147). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -9166,10 +9166,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6242</v>
+        <v>0.609</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-166</v>
+        <v>-156</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>122</v>
@@ -9196,7 +9196,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 62.4% (fair -166). Your call.</t>
+          <t>Model 60.9% (fair -156). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -9741,12 +9741,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Los Angeles Angels @ Minnesota Twins</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -9760,13 +9760,13 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5336000000000001</v>
+        <v>0.5663</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-114</v>
+        <v>-131</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9790,7 +9790,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -114). Your call.</t>
+          <t>Model 56.6% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9817,22 +9817,22 @@
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals -1.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4261</v>
+        <v>0.5336000000000001</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>135</v>
+        <v>-114</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>165</v>
+        <v>112</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9856,7 +9856,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 42.6% (fair +135). Your call.</t>
+          <t>Model 53.4% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9873,32 +9873,32 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever @ Las Vegas Aces</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Over 181.5</t>
+          <t>Washington Nationals -1.5</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5185999999999999</v>
+        <v>0.4261</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-108</v>
+        <v>135</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>113</v>
+        <v>165</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9922,7 +9922,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 42.6% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9939,32 +9939,32 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Indiana Fever @ Las Vegas Aces</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Over 181.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5249</v>
+        <v>0.5197000000000001</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -9988,7 +9988,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 52.5% (fair -110). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -10005,32 +10005,32 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Angels @ Minnesota Twins</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5347</v>
+        <v>0.5249</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 52.5% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10137,32 +10137,32 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Angels @ Minnesota Twins</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5816</v>
+        <v>0.5095</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-139</v>
+        <v>-104</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-122</v>
+        <v>107</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -10186,7 +10186,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -10203,7 +10203,7 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Athletics @ Chicago White Sox</t>
+          <t>Los Angeles Angels @ Minnesota Twins</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
@@ -10213,22 +10213,22 @@
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox -1.5</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4124</v>
+        <v>0.5767</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>142</v>
+        <v>-136</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>156</v>
+        <v>-122</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -10252,7 +10252,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 41.2% (fair +142). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -10288,10 +10288,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4012</v>
+        <v>0.3978</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>163</v>
@@ -10318,7 +10318,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 40.1% (fair +149). Your call.</t>
+          <t>Model 39.8% (fair +151). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -10335,12 +10335,12 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Chicago Sky @ Dallas Wings</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
@@ -10350,17 +10350,17 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Over 8</t>
+          <t>Over 178.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5095</v>
+        <v>0.5125</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-104</v>
+        <v>-105</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -10384,7 +10384,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 51.2% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -10401,26 +10401,26 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Chicago Sky @ Dallas Wings</t>
+          <t>Boston Red Sox @ New York Mets</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Over 178.5</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5125</v>
+        <v>0.512</v>
       </c>
       <c r="G29" s="14" t="n">
         <v>-105</v>
@@ -13795,10 +13795,10 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>0.4184</v>
+        <v>0.4233</v>
       </c>
       <c r="G53" s="14" t="n">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="H53" s="15" t="n">
         <v>122</v>
@@ -13825,7 +13825,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>Model 41.8% (fair +139). Your call.</t>
+          <t>Model 42.3% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O53" s="15" t="n"/>
@@ -13861,10 +13861,10 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.5816</v>
+        <v>0.5767</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>-139</v>
+        <v>-136</v>
       </c>
       <c r="H54" s="15" t="n">
         <v>-122</v>
@@ -13891,7 +13891,7 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O54" s="15" t="n"/>
@@ -13927,10 +13927,10 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.4653</v>
+        <v>0.4337</v>
       </c>
       <c r="G55" s="14" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="H55" s="15" t="n">
         <v>113</v>
@@ -13957,7 +13957,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 43.4% (fair +131). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -13993,10 +13993,10 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.5347</v>
+        <v>0.5663</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>-115</v>
+        <v>-131</v>
       </c>
       <c r="H56" s="15" t="n">
         <v>100</v>
@@ -14023,7 +14023,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 56.6% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -14059,10 +14059,10 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.4012</v>
+        <v>0.3978</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H57" s="15" t="n">
         <v>163</v>
@@ -14089,7 +14089,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 40.1% (fair +149). Your call.</t>
+          <t>Model 39.8% (fair +151). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -14125,10 +14125,10 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.5988</v>
+        <v>0.6022000000000001</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>-149</v>
+        <v>-151</v>
       </c>
       <c r="H58" s="15" t="n">
         <v>-163</v>
@@ -14155,7 +14155,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 59.9% (fair -149). Your call.</t>
+          <t>Model 60.2% (fair -151). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -14323,10 +14323,10 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.6242</v>
+        <v>0.609</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>-166</v>
+        <v>-156</v>
       </c>
       <c r="H61" s="15" t="n">
         <v>122</v>
@@ -14353,7 +14353,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 62.4% (fair -166). Your call.</t>
+          <t>Model 60.9% (fair -156). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -14389,10 +14389,10 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.3758</v>
+        <v>0.391</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="H62" s="15" t="n">
         <v>122</v>
@@ -14419,7 +14419,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 37.6% (fair +166). Your call.</t>
+          <t>Model 39.1% (fair +156). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -14455,10 +14455,10 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>0.4124</v>
+        <v>0.4054</v>
       </c>
       <c r="G63" s="14" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="H63" s="15" t="n">
         <v>156</v>
@@ -14485,7 +14485,7 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>Model 41.2% (fair +142). Your call.</t>
+          <t>Model 40.5% (fair +147). Your call.</t>
         </is>
       </c>
       <c r="O63" s="15" t="n"/>
@@ -14521,10 +14521,10 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.5876</v>
+        <v>0.5946</v>
       </c>
       <c r="G64" s="14" t="n">
-        <v>-142</v>
+        <v>-147</v>
       </c>
       <c r="H64" s="15" t="n">
         <v>178</v>
@@ -14551,7 +14551,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>Model 58.8% (fair -142). Your call.</t>
+          <t>Model 59.5% (fair -147). Your call.</t>
         </is>
       </c>
       <c r="O64" s="15" t="n"/>
@@ -14587,10 +14587,10 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>0.4608</v>
+        <v>0.4645</v>
       </c>
       <c r="G65" s="14" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H65" s="15" t="n"/>
       <c r="I65" s="13">
@@ -14615,7 +14615,7 @@
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 46.5% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O65" s="15" t="n"/>
@@ -14651,10 +14651,10 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>0.5392</v>
+        <v>0.5355</v>
       </c>
       <c r="G66" s="14" t="n">
-        <v>-117</v>
+        <v>-115</v>
       </c>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="13">
@@ -14679,7 +14679,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 53.5% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O66" s="15" t="n"/>
@@ -14715,10 +14715,10 @@
         </is>
       </c>
       <c r="F67" s="13" t="n">
-        <v>0.4079</v>
+        <v>0.4157</v>
       </c>
       <c r="G67" s="14" t="n">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="H67" s="15" t="n"/>
       <c r="I67" s="13">
@@ -14743,7 +14743,7 @@
       </c>
       <c r="N67" s="19" t="inlineStr">
         <is>
-          <t>Model 40.8% (fair +145). Your call.</t>
+          <t>Model 41.6% (fair +141). Your call.</t>
         </is>
       </c>
       <c r="O67" s="15" t="n"/>
@@ -14779,10 +14779,10 @@
         </is>
       </c>
       <c r="F68" s="13" t="n">
-        <v>0.5921</v>
+        <v>0.5843</v>
       </c>
       <c r="G68" s="14" t="n">
-        <v>-145</v>
+        <v>-141</v>
       </c>
       <c r="H68" s="15" t="n"/>
       <c r="I68" s="13">
@@ -14807,7 +14807,7 @@
       </c>
       <c r="N68" s="19" t="inlineStr">
         <is>
-          <t>Model 59.2% (fair -145). Your call.</t>
+          <t>Model 58.4% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O68" s="15" t="n"/>
@@ -14843,10 +14843,10 @@
         </is>
       </c>
       <c r="F69" s="13" t="n">
-        <v>0.4581</v>
+        <v>0.4548</v>
       </c>
       <c r="G69" s="14" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H69" s="15" t="n"/>
       <c r="I69" s="13">
@@ -14871,7 +14871,7 @@
       </c>
       <c r="N69" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +118). Your call.</t>
+          <t>Model 45.5% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O69" s="15" t="n"/>
@@ -14907,10 +14907,10 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>0.5419</v>
+        <v>0.5452</v>
       </c>
       <c r="G70" s="14" t="n">
-        <v>-118</v>
+        <v>-120</v>
       </c>
       <c r="H70" s="15" t="n"/>
       <c r="I70" s="13">
@@ -14935,7 +14935,7 @@
       </c>
       <c r="N70" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O70" s="15" t="n"/>
@@ -14971,7 +14971,7 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>0.4422</v>
+        <v>0.4429</v>
       </c>
       <c r="G71" s="14" t="n">
         <v>126</v>
@@ -14999,7 +14999,7 @@
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>Model 44.2% (fair +126). Your call.</t>
+          <t>Model 44.3% (fair +126). Your call.</t>
         </is>
       </c>
       <c r="O71" s="15" t="n"/>
@@ -15035,7 +15035,7 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.5578</v>
+        <v>0.5571</v>
       </c>
       <c r="G72" s="14" t="n">
         <v>-126</v>
@@ -15063,7 +15063,7 @@
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 55.7% (fair -126). Your call.</t>
         </is>
       </c>
       <c r="O72" s="15" t="n"/>
@@ -15099,10 +15099,10 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.5392</v>
+        <v>0.538</v>
       </c>
       <c r="G73" s="14" t="n">
-        <v>-117</v>
+        <v>-116</v>
       </c>
       <c r="H73" s="15" t="n"/>
       <c r="I73" s="13">
@@ -15127,7 +15127,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 53.8% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O73" s="15" t="n"/>
@@ -15163,10 +15163,10 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.4608</v>
+        <v>0.462</v>
       </c>
       <c r="G74" s="14" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H74" s="15" t="n"/>
       <c r="I74" s="13">
@@ -15191,7 +15191,7 @@
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 46.2% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O74" s="15" t="n"/>
@@ -15374,7 +15374,7 @@
         <v>356</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>400</v>
+        <v>426</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -15440,7 +15440,7 @@
         <v>-356</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -15628,17 +15628,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Dallas Wings -9.5</t>
+          <t>Dallas Wings -11.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5162</v>
+        <v>0.4573601332209344</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-107</v>
+        <v>119</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>-104</v>
+        <v>115</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -15662,7 +15662,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 51.6% (fair -107). Your call.</t>
+          <t>Model 45.7% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -15694,17 +15694,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky +9.5</t>
+          <t>Chicago Sky +11.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.4838</v>
+        <v>0.5426398667790656</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>107</v>
+        <v>-119</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -15728,7 +15728,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 48.4% (fair +107). Your call.</t>
+          <t>Model 54.3% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -15770,7 +15770,7 @@
         <v>150</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>180</v>
+        <v>198</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -15896,7 +15896,7 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5185999999999999</v>
+        <v>0.5197000000000001</v>
       </c>
       <c r="G13" s="14" t="n">
         <v>-108</v>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -15962,13 +15962,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4814000000000001</v>
+        <v>0.4802999999999999</v>
       </c>
       <c r="G14" s="14" t="n">
         <v>108</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-108</v>
+        <v>-106</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -15992,7 +15992,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -16024,17 +16024,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Las Vegas Aces -6</t>
+          <t>Las Vegas Aces -6.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4520544547810846</v>
+        <v>0.4365025644033865</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -16058,7 +16058,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 45.2% (fair +121). Your call.</t>
+          <t>Model 43.7% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -16090,14 +16090,14 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Indiana Fever +6</t>
+          <t>Indiana Fever +6.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5167455452189154</v>
+        <v>0.5634974355966135</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-107</v>
+        <v>-129</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>138</v>
@@ -16124,7 +16124,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 56.3% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -16166,7 +16166,7 @@
         <v>202</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>285</v>
+        <v>317</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -16292,10 +16292,10 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5237000000000001</v>
+        <v>0.5266999999999999</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-110</v>
+        <v>-111</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>-105</v>
@@ -16322,7 +16322,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 52.7% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -16358,13 +16358,13 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4762999999999999</v>
+        <v>0.4733000000000001</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -16388,7 +16388,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 47.3% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -16430,7 +16430,7 @@
         <v>138</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -16562,7 +16562,7 @@
         <v>1157</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>733</v>
+        <v>669</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -17031,22 +17031,22 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="C5" s="22" t="n">
         <v>0.2488</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>598</v>
+        <v>606</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>0.3956</v>
+        <v>0.3904</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>-79.88</v>
+        <v>-87.88</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>-13.45</v>
+        <v>-14.6</v>
       </c>
       <c r="H5" s="24" t="n">
         <v>4.11</v>
@@ -17062,22 +17062,22 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="C6" s="22" t="n">
         <v>0.2497</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>537</v>
+        <v>545</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>0.3921</v>
+        <v>0.3863</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>-77.90000000000001</v>
+        <v>-85.90000000000001</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>-14.62</v>
+        <v>-15.88</v>
       </c>
       <c r="H6" s="24" t="n">
         <v>5.86</v>
@@ -17166,7 +17166,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>When the model said X%, how often it actually happened (n=414, ECE 0.045 — lower is better; a calibrated model's bars sit on the diagonal).</t>
+          <t>When the model said X%, how often it actually happened (n=416, ECE 0.042 — lower is better; a calibrated model's bars sit on the diagonal).</t>
         </is>
       </c>
     </row>
@@ -17261,16 +17261,16 @@
         </is>
       </c>
       <c r="B20" s="21" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C20" s="13" t="n">
-        <v>0.459</v>
+        <v>0.4591</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>0.4297</v>
+        <v>0.4341</v>
       </c>
       <c r="E20" s="26" t="n">
-        <v>-0.0294</v>
+        <v>-0.025</v>
       </c>
     </row>
     <row r="21">
@@ -17280,16 +17280,16 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>0.5431</v>
+        <v>0.5432</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>0.5385</v>
+        <v>0.541</v>
       </c>
       <c r="E21" s="26" t="n">
-        <v>-0.0047</v>
+        <v>-0.0022</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
data: hourly update 2026-07-13 00:07Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-12.xlsx
+++ b/data/output/workbook/2026-07-12.xlsx
@@ -521,7 +521,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="10648950"/>
+    <ext cx="10125075" cy="10496550"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -581,7 +581,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="10582275"/>
+    <ext cx="10125075" cy="10839450"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-12 19:04</t>
+          <t>2026-07-12 20:07</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q82"/>
+  <dimension ref="A1:Q81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3979,167 +3979,246 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="29" t="inlineStr">
+        <is>
+          <t>Seattle Mariners offense vs Tampa Bay Rays defense</t>
+        </is>
+      </c>
+    </row>
     <row r="68">
-      <c r="A68" s="29" t="inlineStr">
-        <is>
-          <t>Seattle Mariners offense vs Tampa Bay Rays defense</t>
+      <c r="A68" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B68" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C68" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D68" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E68" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F68" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G68" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H68" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I68" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J68" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K68" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L68" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M68" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N68" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O68" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P68" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q68" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B69" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C69" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D69" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E69" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F69" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G69" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H69" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I69" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J69" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K69" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L69" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M69" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N69" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O69" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P69" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q69" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A69" s="31" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B69" s="32" t="n">
+        <v>3.853</v>
+      </c>
+      <c r="C69" s="32" t="n">
+        <v>3.533</v>
+      </c>
+      <c r="D69" s="32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E69" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F69" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G69" s="32" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H69" s="34" t="inlineStr">
+        <is>
+          <t>29th</t>
+        </is>
+      </c>
+      <c r="I69" s="32" t="inlineStr"/>
+      <c r="J69" s="36" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="K69" s="32" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="L69" s="32" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="M69" s="32" t="n">
+        <v>3.133</v>
+      </c>
+      <c r="N69" s="32" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="O69" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="P69" s="32" t="n">
+        <v>4.366</v>
+      </c>
+      <c r="Q69" s="35" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="31" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B70" s="32" t="n">
-        <v>3.853</v>
-      </c>
-      <c r="C70" s="32" t="n">
-        <v>3.533</v>
-      </c>
-      <c r="D70" s="32" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="E70" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="F70" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="G70" s="32" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="H70" s="34" t="inlineStr">
-        <is>
-          <t>29th</t>
+        <v>7.854</v>
+      </c>
+      <c r="C70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H70" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="I70" s="32" t="inlineStr"/>
-      <c r="J70" s="36" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="K70" s="32" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="L70" s="32" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="M70" s="32" t="n">
-        <v>3.133</v>
-      </c>
-      <c r="N70" s="32" t="n">
-        <v>3.45</v>
-      </c>
-      <c r="O70" s="32" t="n">
-        <v>3.6</v>
+      <c r="J70" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O70" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="P70" s="32" t="n">
-        <v>4.366</v>
+        <v>8.467000000000001</v>
       </c>
       <c r="Q70" s="35" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>7.854</v>
+        <v>1.312</v>
       </c>
       <c r="C71" s="32" t="inlineStr">
         <is>
@@ -4203,22 +4282,22 @@
         </is>
       </c>
       <c r="P71" s="32" t="n">
-        <v>8.467000000000001</v>
+        <v>1.444</v>
       </c>
       <c r="Q71" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B72" s="32" t="n">
-        <v>1.312</v>
+        <v>8.646000000000001</v>
       </c>
       <c r="C72" s="32" t="inlineStr">
         <is>
@@ -4282,317 +4361,317 @@
         </is>
       </c>
       <c r="P72" s="32" t="n">
-        <v>1.444</v>
+        <v>7.778</v>
       </c>
       <c r="Q72" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B73" s="32" t="n">
-        <v>8.646000000000001</v>
-      </c>
-      <c r="C73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H73" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>0.427</v>
+      </c>
+      <c r="C73" s="32" t="n">
+        <v>0.233</v>
+      </c>
+      <c r="D73" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E73" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="34" t="inlineStr">
+        <is>
+          <t>28th</t>
         </is>
       </c>
       <c r="I73" s="32" t="inlineStr"/>
-      <c r="J73" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O73" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J73" s="36" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="K73" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M73" s="32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N73" s="32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O73" s="32" t="n">
+        <v>0.333</v>
       </c>
       <c r="P73" s="32" t="n">
-        <v>7.778</v>
+        <v>0.463</v>
       </c>
       <c r="Q73" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="31" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B74" s="32" t="n">
-        <v>0.427</v>
-      </c>
-      <c r="C74" s="32" t="n">
-        <v>0.233</v>
-      </c>
-      <c r="D74" s="32" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E74" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F74" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="G74" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H74" s="34" t="inlineStr">
-        <is>
-          <t>28th</t>
-        </is>
-      </c>
-      <c r="I74" s="32" t="inlineStr"/>
-      <c r="J74" s="36" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="K74" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L74" s="32" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="M74" s="32" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="N74" s="32" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="O74" s="32" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="P74" s="32" t="n">
-        <v>0.463</v>
-      </c>
-      <c r="Q74" s="35" t="inlineStr">
-        <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="29" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays offense vs Seattle Mariners defense</t>
+        </is>
+      </c>
+    </row>
     <row r="76">
-      <c r="A76" s="29" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays offense vs Seattle Mariners defense</t>
+      <c r="A76" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B76" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D76" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E76" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F76" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G76" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H76" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I76" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J76" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K76" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L76" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M76" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N76" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O76" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P76" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q76" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B77" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C77" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D77" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E77" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F77" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G77" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H77" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I77" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J77" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K77" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L77" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M77" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N77" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O77" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P77" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q77" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A77" s="31" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B77" s="32" t="n">
+        <v>4.659</v>
+      </c>
+      <c r="C77" s="32" t="n">
+        <v>4.567</v>
+      </c>
+      <c r="D77" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E77" s="32" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F77" s="32" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G77" s="32" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="H77" s="36" t="inlineStr">
+        <is>
+          <t>8th</t>
+        </is>
+      </c>
+      <c r="I77" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J77" s="34" t="inlineStr">
+        <is>
+          <t>24th</t>
+        </is>
+      </c>
+      <c r="K77" s="32" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="L77" s="32" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="M77" s="32" t="n">
+        <v>3.467</v>
+      </c>
+      <c r="N77" s="32" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="O77" s="32" t="n">
+        <v>4.167</v>
+      </c>
+      <c r="P77" s="32" t="n">
+        <v>4.042</v>
+      </c>
+      <c r="Q77" s="35" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B78" s="32" t="n">
-        <v>4.659</v>
-      </c>
-      <c r="C78" s="32" t="n">
-        <v>4.567</v>
-      </c>
-      <c r="D78" s="32" t="n">
-        <v>5</v>
-      </c>
-      <c r="E78" s="32" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="F78" s="32" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="G78" s="32" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="H78" s="36" t="inlineStr">
-        <is>
-          <t>8th</t>
-        </is>
-      </c>
-      <c r="I78" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J78" s="34" t="inlineStr">
-        <is>
-          <t>24th</t>
-        </is>
-      </c>
-      <c r="K78" s="32" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="L78" s="32" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="M78" s="32" t="n">
-        <v>3.467</v>
-      </c>
-      <c r="N78" s="32" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="O78" s="32" t="n">
-        <v>4.167</v>
+        <v>8.778</v>
+      </c>
+      <c r="C78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H78" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I78" s="32" t="inlineStr"/>
+      <c r="J78" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O78" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="P78" s="32" t="n">
-        <v>4.042</v>
+        <v>7.979</v>
       </c>
       <c r="Q78" s="35" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B79" s="32" t="n">
-        <v>8.778</v>
+        <v>0.956</v>
       </c>
       <c r="C79" s="32" t="inlineStr">
         <is>
@@ -4656,22 +4735,22 @@
         </is>
       </c>
       <c r="P79" s="32" t="n">
-        <v>7.979</v>
+        <v>0.958</v>
       </c>
       <c r="Q79" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B80" s="32" t="n">
-        <v>0.956</v>
+        <v>7.244</v>
       </c>
       <c r="C80" s="32" t="inlineStr">
         <is>
@@ -4735,147 +4814,68 @@
         </is>
       </c>
       <c r="P80" s="32" t="n">
-        <v>0.958</v>
+        <v>8.333</v>
       </c>
       <c r="Q80" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B81" s="32" t="n">
-        <v>7.244</v>
-      </c>
-      <c r="C81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H81" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>0.512</v>
+      </c>
+      <c r="C81" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D81" s="32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E81" s="32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F81" s="32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G81" s="32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H81" s="33" t="inlineStr">
+        <is>
+          <t>15th</t>
         </is>
       </c>
       <c r="I81" s="32" t="inlineStr"/>
-      <c r="J81" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O81" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J81" s="33" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="K81" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N81" s="32" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O81" s="32" t="n">
+        <v>0.3</v>
       </c>
       <c r="P81" s="32" t="n">
-        <v>8.333</v>
+        <v>0.378</v>
       </c>
       <c r="Q81" s="35" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="31" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B82" s="32" t="n">
-        <v>0.512</v>
-      </c>
-      <c r="C82" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D82" s="32" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E82" s="32" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F82" s="32" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G82" s="32" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H82" s="33" t="inlineStr">
-        <is>
-          <t>15th</t>
-        </is>
-      </c>
-      <c r="I82" s="32" t="inlineStr"/>
-      <c r="J82" s="33" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="K82" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L82" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M82" s="32" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N82" s="32" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="O82" s="32" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P82" s="32" t="n">
-        <v>0.378</v>
-      </c>
-      <c r="Q82" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -5826,7 +5826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q81"/>
+  <dimension ref="A1:Q83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5843,325 +5843,167 @@
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="29" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="29" t="inlineStr">
         <is>
           <t>Cleveland Guardians offense vs Miami Marlins defense</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="30" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B68" s="30" t="inlineStr">
+      <c r="B70" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C68" s="30" t="inlineStr">
+      <c r="C70" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D68" s="30" t="inlineStr">
+      <c r="D70" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E68" s="30" t="inlineStr">
+      <c r="E70" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F68" s="30" t="inlineStr">
+      <c r="F70" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G68" s="30" t="inlineStr">
+      <c r="G70" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H68" s="30" t="inlineStr">
+      <c r="H70" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I68" s="30" t="inlineStr">
+      <c r="I70" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J68" s="30" t="inlineStr">
+      <c r="J70" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K68" s="30" t="inlineStr">
+      <c r="K70" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L68" s="30" t="inlineStr">
+      <c r="L70" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M68" s="30" t="inlineStr">
+      <c r="M70" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N68" s="30" t="inlineStr">
+      <c r="N70" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O68" s="30" t="inlineStr">
+      <c r="O70" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P68" s="30" t="inlineStr">
+      <c r="P70" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q68" s="30" t="inlineStr">
+      <c r="Q70" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B69" s="32" t="n">
-        <v>3.919</v>
-      </c>
-      <c r="C69" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="D69" s="32" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="E69" s="32" t="n">
-        <v>4</v>
-      </c>
-      <c r="F69" s="32" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="G69" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="H69" s="34" t="inlineStr">
-        <is>
-          <t>25th</t>
-        </is>
-      </c>
-      <c r="I69" s="32" t="inlineStr"/>
-      <c r="J69" s="36" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="K69" s="32" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="L69" s="32" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="M69" s="32" t="n">
-        <v>4.267</v>
-      </c>
-      <c r="N69" s="32" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="O69" s="32" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="P69" s="32" t="n">
-        <v>4.271</v>
-      </c>
-      <c r="Q69" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="31" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B70" s="32" t="n">
-        <v>7.735</v>
-      </c>
-      <c r="C70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I70" s="32" t="inlineStr"/>
-      <c r="J70" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O70" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P70" s="32" t="n">
-        <v>7.694</v>
-      </c>
-      <c r="Q70" s="35" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>0.959</v>
-      </c>
-      <c r="C71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H71" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>3.919</v>
+      </c>
+      <c r="C71" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D71" s="32" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="E71" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F71" s="32" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G71" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H71" s="34" t="inlineStr">
+        <is>
+          <t>25th</t>
         </is>
       </c>
       <c r="I71" s="32" t="inlineStr"/>
-      <c r="J71" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O71" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J71" s="36" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="K71" s="32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L71" s="32" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="M71" s="32" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="N71" s="32" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="O71" s="32" t="n">
+        <v>3.8</v>
       </c>
       <c r="P71" s="32" t="n">
-        <v>1.082</v>
+        <v>4.271</v>
       </c>
       <c r="Q71" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B72" s="32" t="n">
-        <v>8</v>
+        <v>7.735</v>
       </c>
       <c r="C72" s="32" t="inlineStr">
         <is>
@@ -6225,392 +6067,392 @@
         </is>
       </c>
       <c r="P72" s="32" t="n">
-        <v>8.531000000000001</v>
+        <v>7.694</v>
       </c>
       <c r="Q72" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
         <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B73" s="32" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="C73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="inlineStr"/>
+      <c r="J73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P73" s="32" t="n">
+        <v>1.082</v>
+      </c>
+      <c r="Q73" s="35" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="31" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B74" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H74" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I74" s="32" t="inlineStr"/>
+      <c r="J74" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O74" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P74" s="32" t="n">
+        <v>8.531000000000001</v>
+      </c>
+      <c r="Q74" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B73" s="32" t="n">
+      <c r="B75" s="32" t="n">
         <v>0.494</v>
       </c>
-      <c r="C73" s="32" t="n">
+      <c r="C75" s="32" t="n">
         <v>0.267</v>
       </c>
-      <c r="D73" s="32" t="n">
+      <c r="D75" s="32" t="n">
         <v>0.35</v>
       </c>
-      <c r="E73" s="32" t="n">
+      <c r="E75" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="F73" s="32" t="n">
+      <c r="F75" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="G73" s="32" t="n">
+      <c r="G75" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H73" s="34" t="inlineStr">
+      <c r="H75" s="34" t="inlineStr">
         <is>
           <t>29th</t>
         </is>
       </c>
-      <c r="I73" s="32" t="inlineStr"/>
-      <c r="J73" s="36" t="inlineStr">
+      <c r="I75" s="32" t="inlineStr"/>
+      <c r="J75" s="36" t="inlineStr">
         <is>
           <t>3rd</t>
         </is>
       </c>
-      <c r="K73" s="32" t="n">
+      <c r="K75" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="L73" s="32" t="n">
+      <c r="L75" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="M73" s="32" t="n">
+      <c r="M75" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="N73" s="32" t="n">
+      <c r="N75" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="O73" s="32" t="n">
+      <c r="O75" s="32" t="n">
         <v>0.333</v>
       </c>
-      <c r="P73" s="32" t="n">
+      <c r="P75" s="32" t="n">
         <v>0.578</v>
       </c>
-      <c r="Q73" s="35" t="inlineStr">
+      <c r="Q75" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="29" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="29" t="inlineStr">
         <is>
           <t>Miami Marlins offense vs Cleveland Guardians defense</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="30" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="30" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B76" s="30" t="inlineStr">
+      <c r="B78" s="30" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C76" s="30" t="inlineStr">
+      <c r="C78" s="30" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D76" s="30" t="inlineStr">
+      <c r="D78" s="30" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E76" s="30" t="inlineStr">
+      <c r="E78" s="30" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F76" s="30" t="inlineStr">
+      <c r="F78" s="30" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G76" s="30" t="inlineStr">
+      <c r="G78" s="30" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H76" s="30" t="inlineStr">
+      <c r="H78" s="30" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I76" s="30" t="inlineStr">
+      <c r="I78" s="30" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J76" s="30" t="inlineStr">
+      <c r="J78" s="30" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K76" s="30" t="inlineStr">
+      <c r="K78" s="30" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L76" s="30" t="inlineStr">
+      <c r="L78" s="30" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M76" s="30" t="inlineStr">
+      <c r="M78" s="30" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N76" s="30" t="inlineStr">
+      <c r="N78" s="30" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O76" s="30" t="inlineStr">
+      <c r="O78" s="30" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P76" s="30" t="inlineStr">
+      <c r="P78" s="30" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q76" s="30" t="inlineStr">
+      <c r="Q78" s="30" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="31" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B77" s="32" t="n">
-        <v>4.647</v>
-      </c>
-      <c r="C77" s="32" t="n">
-        <v>5.367</v>
-      </c>
-      <c r="D77" s="32" t="n">
-        <v>5.45</v>
-      </c>
-      <c r="E77" s="32" t="n">
-        <v>5.867</v>
-      </c>
-      <c r="F77" s="32" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="G77" s="32" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="H77" s="33" t="inlineStr">
-        <is>
-          <t>20th</t>
-        </is>
-      </c>
-      <c r="I77" s="32" t="inlineStr"/>
-      <c r="J77" s="36" t="inlineStr">
-        <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="K77" s="32" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="L77" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="M77" s="32" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="N77" s="32" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="O77" s="32" t="n">
-        <v>4.133</v>
-      </c>
-      <c r="P77" s="32" t="n">
-        <v>4.07</v>
-      </c>
-      <c r="Q77" s="35" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="31" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B78" s="32" t="n">
-        <v>8.286</v>
-      </c>
-      <c r="C78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H78" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I78" s="32" t="inlineStr"/>
-      <c r="J78" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O78" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P78" s="32" t="n">
-        <v>7.939</v>
-      </c>
-      <c r="Q78" s="35" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B79" s="32" t="n">
-        <v>0.918</v>
-      </c>
-      <c r="C79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H79" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
+        <v>4.647</v>
+      </c>
+      <c r="C79" s="32" t="n">
+        <v>5.367</v>
+      </c>
+      <c r="D79" s="32" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="E79" s="32" t="n">
+        <v>5.867</v>
+      </c>
+      <c r="F79" s="32" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="G79" s="32" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H79" s="33" t="inlineStr">
+        <is>
+          <t>20th</t>
         </is>
       </c>
       <c r="I79" s="32" t="inlineStr"/>
-      <c r="J79" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O79" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J79" s="36" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="K79" s="32" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L79" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M79" s="32" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N79" s="32" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="O79" s="32" t="n">
+        <v>4.133</v>
       </c>
       <c r="P79" s="32" t="n">
-        <v>1.143</v>
+        <v>4.07</v>
       </c>
       <c r="Q79" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B80" s="32" t="n">
-        <v>7.816</v>
+        <v>8.286</v>
       </c>
       <c r="C80" s="32" t="inlineStr">
         <is>
@@ -6674,68 +6516,226 @@
         </is>
       </c>
       <c r="P80" s="32" t="n">
-        <v>9.388</v>
+        <v>7.939</v>
       </c>
       <c r="Q80" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
         <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B81" s="32" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="C81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I81" s="32" t="inlineStr"/>
+      <c r="J81" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O81" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P81" s="32" t="n">
+        <v>1.143</v>
+      </c>
+      <c r="Q81" s="35" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="31" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B82" s="32" t="n">
+        <v>7.816</v>
+      </c>
+      <c r="C82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H82" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I82" s="32" t="inlineStr"/>
+      <c r="J82" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O82" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P82" s="32" t="n">
+        <v>9.388</v>
+      </c>
+      <c r="Q82" s="35" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="31" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B81" s="32" t="n">
+      <c r="B83" s="32" t="n">
         <v>0.578</v>
       </c>
-      <c r="C81" s="32" t="n">
+      <c r="C83" s="32" t="n">
         <v>0.5669999999999999</v>
       </c>
-      <c r="D81" s="32" t="n">
+      <c r="D83" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="E81" s="32" t="n">
+      <c r="E83" s="32" t="n">
         <v>0.733</v>
       </c>
-      <c r="F81" s="32" t="n">
+      <c r="F83" s="32" t="n">
         <v>0.9</v>
       </c>
-      <c r="G81" s="32" t="n">
+      <c r="G83" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="H81" s="34" t="inlineStr">
+      <c r="H83" s="34" t="inlineStr">
         <is>
           <t>21st</t>
         </is>
       </c>
-      <c r="I81" s="32" t="inlineStr"/>
-      <c r="J81" s="33" t="inlineStr">
+      <c r="I83" s="32" t="inlineStr"/>
+      <c r="J83" s="33" t="inlineStr">
         <is>
           <t>12th</t>
         </is>
       </c>
-      <c r="K81" s="32" t="n">
+      <c r="K83" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="L81" s="32" t="n">
+      <c r="L83" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="M81" s="32" t="n">
+      <c r="M83" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="N81" s="32" t="n">
+      <c r="N83" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="O81" s="32" t="n">
+      <c r="O83" s="32" t="n">
         <v>0.433</v>
       </c>
-      <c r="P81" s="32" t="n">
+      <c r="P83" s="32" t="n">
         <v>0.361</v>
       </c>
-      <c r="Q81" s="35" t="inlineStr">
+      <c r="Q83" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -8836,10 +8836,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6608000000000001</v>
+        <v>0.6557999999999999</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-195</v>
+        <v>-191</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>186</v>
@@ -8866,7 +8866,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 66.1% (fair -195). Your call.</t>
+          <t>Model 65.6% (fair -191). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -8902,10 +8902,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5946</v>
+        <v>0.5911</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-147</v>
+        <v>-145</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>178</v>
@@ -8932,7 +8932,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 59.5% (fair -147). Your call.</t>
+          <t>Model 59.1% (fair -145). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -8949,12 +8949,12 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -8964,17 +8964,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Cleveland Guardians +1.5</t>
+          <t>Milwaukee Brewers +1.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.601</v>
+        <v>0.5674</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-151</v>
+        <v>-131</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -8998,7 +8998,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 60.1% (fair -151). Your call.</t>
+          <t>Model 56.7% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -9015,12 +9015,12 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers @ Pittsburgh Pirates</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -9030,17 +9030,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers +1.5</t>
+          <t>Cleveland Guardians +1.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5660000000000001</v>
+        <v>0.5974999999999999</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-130</v>
+        <v>-148</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -9064,7 +9064,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 56.6% (fair -130). Your call.</t>
+          <t>Model 59.7% (fair -148). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -9100,10 +9100,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5739000000000001</v>
+        <v>0.5796</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-135</v>
+        <v>-138</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>170</v>
@@ -9130,7 +9130,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 57.4% (fair -135). Your call.</t>
+          <t>Model 58.0% (fair -138). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -9166,10 +9166,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.609</v>
+        <v>0.622</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-156</v>
+        <v>-165</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>122</v>
@@ -9196,7 +9196,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -156). Your call.</t>
+          <t>Model 62.2% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -9213,12 +9213,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies @ Detroit Tigers</t>
+          <t>Kansas City Royals @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -9228,17 +9228,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5655</v>
+        <v>0.5637</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-130</v>
+        <v>-129</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -9262,7 +9262,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 56.5% (fair -130). Your call.</t>
+          <t>Model 56.4% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -9345,12 +9345,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Kansas City Royals @ Baltimore Orioles</t>
+          <t>Philadelphia Phillies @ Detroit Tigers</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -9360,17 +9360,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5575</v>
+        <v>0.5641</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-126</v>
+        <v>-129</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -9394,7 +9394,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 56.4% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -9430,10 +9430,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5501</v>
+        <v>0.5706</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-122</v>
+        <v>-133</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>122</v>
@@ -9460,7 +9460,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 57.1% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -9487,22 +9487,22 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Pittsburgh Pirates -1.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5725</v>
+        <v>0.4326</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-134</v>
+        <v>131</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>111</v>
+        <v>178</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -9526,7 +9526,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 57.2% (fair -134). Your call.</t>
+          <t>Model 43.3% (fair +131). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -9553,22 +9553,22 @@
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates -1.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.434</v>
+        <v>0.5698</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>130</v>
+        <v>-132</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>178</v>
+        <v>111</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -9592,7 +9592,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 43.4% (fair +130). Your call.</t>
+          <t>Model 57.0% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -9694,10 +9694,10 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.399</v>
+        <v>0.4025</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>185</v>
@@ -9724,7 +9724,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 39.9% (fair +151). Your call.</t>
+          <t>Model 40.2% (fair +148). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9741,12 +9741,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Angels @ Minnesota Twins</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -9760,13 +9760,13 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5663</v>
+        <v>0.5405</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-131</v>
+        <v>-118</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9790,7 +9790,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 56.6% (fair -131). Your call.</t>
+          <t>Model 54.0% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9817,22 +9817,22 @@
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Washington Nationals -1.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5336000000000001</v>
+        <v>0.4204</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-114</v>
+        <v>138</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>112</v>
+        <v>165</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9856,7 +9856,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -114). Your call.</t>
+          <t>Model 42.0% (fair +138). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9873,32 +9873,32 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals -1.5</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4261</v>
+        <v>0.5362</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>135</v>
+        <v>-116</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>165</v>
+        <v>107</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9922,7 +9922,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 42.6% (fair +135). Your call.</t>
+          <t>Model 53.6% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9954,17 +9954,17 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Over 181.5</t>
+          <t>Over 181</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5197000000000001</v>
+        <v>0.5217000000000001</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-108</v>
+        <v>-109</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -9988,7 +9988,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -108). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -10000,37 +10000,37 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Los Angeles Sparks @ Atlanta Dream</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Los Angeles Sparks +7.5</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5249</v>
+        <v>0.5114000000000001</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 52.5% (fair -110). Your call.</t>
+          <t>Model 51.1% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10071,7 +10071,7 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs @ Cincinnati Reds</t>
+          <t>Cleveland Guardians @ Miami Marlins</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
@@ -10081,22 +10081,22 @@
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs -1.5</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.4628</v>
+        <v>0.5249</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>116</v>
+        <v>-110</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>130</v>
+        <v>104</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10120,7 +10120,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 46.3% (fair +116). Your call.</t>
+          <t>Model 52.5% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10137,7 +10137,7 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Cleveland Guardians @ Miami Marlins</t>
+          <t>Chicago Cubs @ Cincinnati Reds</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
@@ -10147,22 +10147,22 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 8</t>
+          <t>Chicago Cubs -1.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5095</v>
+        <v>0.4628</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-104</v>
+        <v>116</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -10186,7 +10186,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 46.3% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -10222,10 +10222,10 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5767</v>
+        <v>0.581</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-136</v>
+        <v>-139</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>-122</v>
@@ -10252,7 +10252,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 58.1% (fair -139). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -10288,10 +10288,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.3978</v>
+        <v>0.4006</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>163</v>
@@ -10318,7 +10318,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 39.8% (fair +151). Your call.</t>
+          <t>Model 40.1% (fair +150). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -10335,12 +10335,12 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky @ Dallas Wings</t>
+          <t>Los Angeles Angels @ Minnesota Twins</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
@@ -10350,17 +10350,17 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Over 178.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5125</v>
+        <v>0.5266999999999999</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-105</v>
+        <v>-111</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -10384,7 +10384,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 52.7% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -10401,32 +10401,32 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Boston Red Sox @ New York Mets</t>
+          <t>Athletics @ Chicago White Sox</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Chicago White Sox -1.5</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.512</v>
+        <v>0.4089</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-105</v>
+        <v>145</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>104</v>
+        <v>156</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 40.9% (fair +145). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -10627,10 +10627,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4351</v>
+        <v>0.4306</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>118</v>
@@ -10657,7 +10657,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 43.5% (fair +130). Your call.</t>
+          <t>Model 43.1% (fair +132). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -10693,10 +10693,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5649</v>
+        <v>0.5694</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-130</v>
+        <v>-132</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>-120</v>
@@ -10723,7 +10723,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 56.5% (fair -130). Your call.</t>
+          <t>Model 56.9% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -10759,10 +10759,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5725</v>
+        <v>0.5698</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-134</v>
+        <v>-132</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>111</v>
@@ -10789,7 +10789,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 57.2% (fair -134). Your call.</t>
+          <t>Model 57.0% (fair -132). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -10825,10 +10825,10 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4275</v>
+        <v>0.4302</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>-102</v>
@@ -10855,7 +10855,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 42.8% (fair +134). Your call.</t>
+          <t>Model 43.0% (fair +132). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -10891,10 +10891,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.434</v>
+        <v>0.4326</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>178</v>
@@ -10921,7 +10921,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 43.4% (fair +130). Your call.</t>
+          <t>Model 43.3% (fair +131). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -10957,10 +10957,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5660000000000001</v>
+        <v>0.5674</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-130</v>
+        <v>-131</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>178</v>
@@ -10987,7 +10987,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 56.6% (fair -130). Your call.</t>
+          <t>Model 56.7% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -11155,10 +11155,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4425</v>
+        <v>0.4363</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>100</v>
@@ -11185,7 +11185,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 44.2% (fair +126). Your call.</t>
+          <t>Model 43.6% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -11221,10 +11221,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5575</v>
+        <v>0.5637</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-126</v>
+        <v>-129</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>129</v>
@@ -11251,7 +11251,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 56.4% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -11287,7 +11287,7 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.422</v>
+        <v>0.4217</v>
       </c>
       <c r="G15" s="14" t="n">
         <v>137</v>
@@ -11353,7 +11353,7 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5780000000000001</v>
+        <v>0.5783</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>-137</v>
@@ -11419,10 +11419,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4471000000000001</v>
+        <v>0.4505</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>115</v>
@@ -11449,7 +11449,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 44.7% (fair +124). Your call.</t>
+          <t>Model 45.1% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -11485,10 +11485,10 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5528999999999999</v>
+        <v>0.5495</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-124</v>
+        <v>-122</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>-113</v>
@@ -11515,7 +11515,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -11551,10 +11551,10 @@
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.4664</v>
+        <v>0.4595</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="H19" s="15" t="n">
         <v>108</v>
@@ -11581,7 +11581,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 46.6% (fair +114). Your call.</t>
+          <t>Model 46.0% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -11617,10 +11617,10 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5336000000000001</v>
+        <v>0.5405</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-114</v>
+        <v>-118</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>112</v>
@@ -11647,7 +11647,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -114). Your call.</t>
+          <t>Model 54.0% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -11683,10 +11683,10 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4261</v>
+        <v>0.4204</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="H21" s="15" t="n">
         <v>165</v>
@@ -11713,7 +11713,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 42.6% (fair +135). Your call.</t>
+          <t>Model 42.0% (fair +138). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -11749,10 +11749,10 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5739000000000001</v>
+        <v>0.5796</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-135</v>
+        <v>-138</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>170</v>
@@ -11779,7 +11779,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 57.4% (fair -135). Your call.</t>
+          <t>Model 58.0% (fair -138). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -12211,7 +12211,7 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.488</v>
+        <v>0.4877</v>
       </c>
       <c r="G29" s="14" t="n">
         <v>105</v>
@@ -12277,7 +12277,7 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.512</v>
+        <v>0.5123</v>
       </c>
       <c r="G30" s="14" t="n">
         <v>-105</v>
@@ -12343,10 +12343,10 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.4499</v>
+        <v>0.4294</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>122</v>
@@ -12373,7 +12373,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 45.0% (fair +122). Your call.</t>
+          <t>Model 42.9% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -12409,10 +12409,10 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.5501</v>
+        <v>0.5706</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>-122</v>
+        <v>-133</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>122</v>
@@ -12439,7 +12439,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 57.1% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -12475,10 +12475,10 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.6212</v>
+        <v>0.6226</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>-164</v>
+        <v>-165</v>
       </c>
       <c r="H33" s="15" t="n">
         <v>-156</v>
@@ -12505,7 +12505,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 62.1% (fair -164). Your call.</t>
+          <t>Model 62.3% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -12541,10 +12541,10 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.3788</v>
+        <v>0.3774</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H34" s="15" t="n">
         <v>156</v>
@@ -12571,7 +12571,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 37.9% (fair +164). Your call.</t>
+          <t>Model 37.7% (fair +165). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -13135,10 +13135,10 @@
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>0.5655</v>
+        <v>0.5641</v>
       </c>
       <c r="G43" s="14" t="n">
-        <v>-130</v>
+        <v>-129</v>
       </c>
       <c r="H43" s="15" t="n">
         <v>127</v>
@@ -13165,7 +13165,7 @@
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>Model 56.5% (fair -130). Your call.</t>
+          <t>Model 56.4% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O43" s="15" t="n"/>
@@ -13201,10 +13201,10 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4345</v>
+        <v>0.4359</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H44" s="15" t="n">
         <v>105</v>
@@ -13231,7 +13231,7 @@
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>Model 43.5% (fair +130). Your call.</t>
+          <t>Model 43.6% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O44" s="15" t="n"/>
@@ -13267,10 +13267,10 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.3392</v>
+        <v>0.3442</v>
       </c>
       <c r="G45" s="14" t="n">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="H45" s="15" t="n">
         <v>186</v>
@@ -13297,7 +13297,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 33.9% (fair +195). Your call.</t>
+          <t>Model 34.4% (fair +191). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -13333,10 +13333,10 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.6608000000000001</v>
+        <v>0.6557999999999999</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>-195</v>
+        <v>-191</v>
       </c>
       <c r="H46" s="15" t="n">
         <v>186</v>
@@ -13363,7 +13363,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 66.1% (fair -195). Your call.</t>
+          <t>Model 65.6% (fair -191). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -13531,10 +13531,10 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>0.5095</v>
+        <v>0.5362</v>
       </c>
       <c r="G49" s="14" t="n">
-        <v>-104</v>
+        <v>-116</v>
       </c>
       <c r="H49" s="15" t="n">
         <v>107</v>
@@ -13561,7 +13561,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 53.6% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O49" s="15" t="n"/>
@@ -13597,10 +13597,10 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.3983</v>
+        <v>0.3723</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="H50" s="15" t="n">
         <v>104</v>
@@ -13627,7 +13627,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>Model 39.8% (fair +151). Your call.</t>
+          <t>Model 37.2% (fair +169). Your call.</t>
         </is>
       </c>
       <c r="O50" s="15" t="n"/>
@@ -13663,10 +13663,10 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>0.399</v>
+        <v>0.4025</v>
       </c>
       <c r="G51" s="14" t="n">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H51" s="15" t="n">
         <v>185</v>
@@ -13693,7 +13693,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>Model 39.9% (fair +151). Your call.</t>
+          <t>Model 40.2% (fair +148). Your call.</t>
         </is>
       </c>
       <c r="O51" s="15" t="n"/>
@@ -13729,10 +13729,10 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.601</v>
+        <v>0.5974999999999999</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>-151</v>
+        <v>-148</v>
       </c>
       <c r="H52" s="15" t="n">
         <v>163</v>
@@ -13759,7 +13759,7 @@
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>Model 60.1% (fair -151). Your call.</t>
+          <t>Model 59.7% (fair -148). Your call.</t>
         </is>
       </c>
       <c r="O52" s="15" t="n"/>
@@ -13795,10 +13795,10 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>0.4233</v>
+        <v>0.419</v>
       </c>
       <c r="G53" s="14" t="n">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H53" s="15" t="n">
         <v>122</v>
@@ -13825,7 +13825,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 41.9% (fair +139). Your call.</t>
         </is>
       </c>
       <c r="O53" s="15" t="n"/>
@@ -13861,10 +13861,10 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.5767</v>
+        <v>0.581</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>-136</v>
+        <v>-139</v>
       </c>
       <c r="H54" s="15" t="n">
         <v>-122</v>
@@ -13891,7 +13891,7 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 58.1% (fair -139). Your call.</t>
         </is>
       </c>
       <c r="O54" s="15" t="n"/>
@@ -13927,10 +13927,10 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.4337</v>
+        <v>0.4733</v>
       </c>
       <c r="G55" s="14" t="n">
-        <v>131</v>
+        <v>111</v>
       </c>
       <c r="H55" s="15" t="n">
         <v>113</v>
@@ -13957,7 +13957,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 43.4% (fair +131). Your call.</t>
+          <t>Model 47.3% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -13993,10 +13993,10 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.5663</v>
+        <v>0.5266999999999999</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>-131</v>
+        <v>-111</v>
       </c>
       <c r="H56" s="15" t="n">
         <v>100</v>
@@ -14023,7 +14023,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 56.6% (fair -131). Your call.</t>
+          <t>Model 52.7% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -14059,10 +14059,10 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.3978</v>
+        <v>0.4006</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H57" s="15" t="n">
         <v>163</v>
@@ -14089,7 +14089,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 39.8% (fair +151). Your call.</t>
+          <t>Model 40.1% (fair +150). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -14125,10 +14125,10 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.6022000000000001</v>
+        <v>0.5993999999999999</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>-151</v>
+        <v>-150</v>
       </c>
       <c r="H58" s="15" t="n">
         <v>-163</v>
@@ -14155,7 +14155,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 60.2% (fair -151). Your call.</t>
+          <t>Model 59.9% (fair -150). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -14323,10 +14323,10 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.609</v>
+        <v>0.622</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>-156</v>
+        <v>-165</v>
       </c>
       <c r="H61" s="15" t="n">
         <v>122</v>
@@ -14353,7 +14353,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -156). Your call.</t>
+          <t>Model 62.2% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -14389,10 +14389,10 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.391</v>
+        <v>0.378</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="H62" s="15" t="n">
         <v>122</v>
@@ -14419,7 +14419,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 39.1% (fair +156). Your call.</t>
+          <t>Model 37.8% (fair +165). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -14455,10 +14455,10 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>0.4054</v>
+        <v>0.4089</v>
       </c>
       <c r="G63" s="14" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H63" s="15" t="n">
         <v>156</v>
@@ -14485,7 +14485,7 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>Model 40.5% (fair +147). Your call.</t>
+          <t>Model 40.9% (fair +145). Your call.</t>
         </is>
       </c>
       <c r="O63" s="15" t="n"/>
@@ -14521,10 +14521,10 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.5946</v>
+        <v>0.5911</v>
       </c>
       <c r="G64" s="14" t="n">
-        <v>-147</v>
+        <v>-145</v>
       </c>
       <c r="H64" s="15" t="n">
         <v>178</v>
@@ -14551,7 +14551,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>Model 59.5% (fair -147). Your call.</t>
+          <t>Model 59.1% (fair -145). Your call.</t>
         </is>
       </c>
       <c r="O64" s="15" t="n"/>
@@ -14587,10 +14587,10 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>0.4645</v>
+        <v>0.4638</v>
       </c>
       <c r="G65" s="14" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H65" s="15" t="n"/>
       <c r="I65" s="13">
@@ -14615,7 +14615,7 @@
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 46.4% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O65" s="15" t="n"/>
@@ -14651,10 +14651,10 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>0.5355</v>
+        <v>0.5362</v>
       </c>
       <c r="G66" s="14" t="n">
-        <v>-115</v>
+        <v>-116</v>
       </c>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="13">
@@ -14679,7 +14679,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 53.6% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O66" s="15" t="n"/>
@@ -14843,10 +14843,10 @@
         </is>
       </c>
       <c r="F69" s="13" t="n">
-        <v>0.4548</v>
+        <v>0.4579</v>
       </c>
       <c r="G69" s="14" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H69" s="15" t="n"/>
       <c r="I69" s="13">
@@ -14871,7 +14871,7 @@
       </c>
       <c r="N69" s="19" t="inlineStr">
         <is>
-          <t>Model 45.5% (fair +120). Your call.</t>
+          <t>Model 45.8% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O69" s="15" t="n"/>
@@ -14907,10 +14907,10 @@
         </is>
       </c>
       <c r="F70" s="13" t="n">
-        <v>0.5452</v>
+        <v>0.5421</v>
       </c>
       <c r="G70" s="14" t="n">
-        <v>-120</v>
+        <v>-118</v>
       </c>
       <c r="H70" s="15" t="n"/>
       <c r="I70" s="13">
@@ -14935,7 +14935,7 @@
       </c>
       <c r="N70" s="19" t="inlineStr">
         <is>
-          <t>Model 54.5% (fair -120). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O70" s="15" t="n"/>
@@ -14971,10 +14971,10 @@
         </is>
       </c>
       <c r="F71" s="13" t="n">
-        <v>0.4429</v>
+        <v>0.4479</v>
       </c>
       <c r="G71" s="14" t="n">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="H71" s="15" t="n"/>
       <c r="I71" s="13">
@@ -14999,7 +14999,7 @@
       </c>
       <c r="N71" s="19" t="inlineStr">
         <is>
-          <t>Model 44.3% (fair +126). Your call.</t>
+          <t>Model 44.8% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O71" s="15" t="n"/>
@@ -15035,10 +15035,10 @@
         </is>
       </c>
       <c r="F72" s="13" t="n">
-        <v>0.5571</v>
+        <v>0.5521</v>
       </c>
       <c r="G72" s="14" t="n">
-        <v>-126</v>
+        <v>-123</v>
       </c>
       <c r="H72" s="15" t="n"/>
       <c r="I72" s="13">
@@ -15063,7 +15063,7 @@
       </c>
       <c r="N72" s="19" t="inlineStr">
         <is>
-          <t>Model 55.7% (fair -126). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O72" s="15" t="n"/>
@@ -15099,10 +15099,10 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.538</v>
+        <v>0.5542</v>
       </c>
       <c r="G73" s="14" t="n">
-        <v>-116</v>
+        <v>-124</v>
       </c>
       <c r="H73" s="15" t="n"/>
       <c r="I73" s="13">
@@ -15127,7 +15127,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Model 53.8% (fair -116). Your call.</t>
+          <t>Model 55.4% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O73" s="15" t="n"/>
@@ -15163,10 +15163,10 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.462</v>
+        <v>0.4458</v>
       </c>
       <c r="G74" s="14" t="n">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="H74" s="15" t="n"/>
       <c r="I74" s="13">
@@ -15191,7 +15191,7 @@
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>Model 46.2% (fair +116). Your call.</t>
+          <t>Model 44.6% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O74" s="15" t="n"/>
@@ -15440,7 +15440,7 @@
         <v>-356</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-110</v>
+        <v>-120</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -15704,7 +15704,7 @@
         <v>-119</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -15770,7 +15770,7 @@
         <v>150</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -15892,17 +15892,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 181.5</t>
+          <t>Over 181</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5197000000000001</v>
+        <v>0.5217000000000001</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-108</v>
+        <v>-109</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -15926,7 +15926,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -108). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -15958,17 +15958,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 181.5</t>
+          <t>Under 181</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4802999999999999</v>
+        <v>0.4551999999999999</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -15992,7 +15992,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 45.5% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -16288,17 +16288,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 180.5</t>
+          <t>Over 179.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5266999999999999</v>
+        <v>0.5549727689112931</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-111</v>
+        <v>-125</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -16322,7 +16322,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 52.7% (fair -111). Your call.</t>
+          <t>Model 55.5% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -16354,17 +16354,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 180.5</t>
+          <t>Under 179.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4733000000000001</v>
+        <v>0.4450272310887069</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -16388,7 +16388,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 47.3% (fair +111). Your call.</t>
+          <t>Model 44.5% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -16420,17 +16420,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream -8.5</t>
+          <t>Atlanta Dream -7.5</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4210482224080958</v>
+        <v>0.4886</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>138</v>
+        <v>105</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>117</v>
+        <v>-108</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -16454,7 +16454,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 42.1% (fair +138). Your call.</t>
+          <t>Model 48.9% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -16486,14 +16486,14 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks +8.5</t>
+          <t>Los Angeles Sparks +7.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5789517775919042</v>
+        <v>0.5114000000000001</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-138</v>
+        <v>-105</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>113</v>
@@ -16520,7 +16520,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 57.9% (fair -138). Your call.</t>
+          <t>Model 51.1% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -16820,10 +16820,10 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.486</v>
+        <v>0.4885</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H27" s="15" t="n">
         <v>-106</v>
@@ -16850,7 +16850,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 48.6% (fair +106). Your call.</t>
+          <t>Model 48.9% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -16886,13 +16886,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.514</v>
+        <v>0.5115000000000001</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -16916,7 +16916,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 51.4% (fair -106). Your call.</t>
+          <t>Model 51.2% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -17031,22 +17031,22 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>0.2488</v>
+        <v>0.249</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>0.3904</v>
+        <v>0.3888</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>-87.88</v>
+        <v>-91.23999999999999</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>-14.6</v>
+        <v>-15.03</v>
       </c>
       <c r="H5" s="24" t="n">
         <v>4.11</v>
@@ -17062,22 +17062,22 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>0.2497</v>
+        <v>0.2498</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>0.3863</v>
+        <v>0.3846</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>-85.90000000000001</v>
+        <v>-89.26000000000001</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>-15.88</v>
+        <v>-16.35</v>
       </c>
       <c r="H6" s="24" t="n">
         <v>5.86</v>
@@ -17166,7 +17166,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>When the model said X%, how often it actually happened (n=416, ECE 0.042 — lower is better; a calibrated model's bars sit on the diagonal).</t>
+          <t>When the model said X%, how often it actually happened (n=417, ECE 0.043 — lower is better; a calibrated model's bars sit on the diagonal).</t>
         </is>
       </c>
     </row>
@@ -17280,16 +17280,16 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>0.5432</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>0.541</v>
+        <v>0.538</v>
       </c>
       <c r="E21" s="26" t="n">
-        <v>-0.0022</v>
+        <v>-0.0052</v>
       </c>
     </row>
     <row r="22">

</xml_diff>